<commit_message>
Added project to export UD_CustomDevice configs from esp to excel
 - moved shared code to separate project
</commit_message>
<xml_diff>
--- a/UD_Modifiers.EspToExcel/Data/UD_Empty.xlsx
+++ b/UD_Modifiers.EspToExcel/Data/UD_Empty.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DEVELOP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DEVELOP\[UD]\[Synth]\Synthesis.UDPatches\UD_Modifiers.EspToExcel\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -20,7 +20,7 @@
     <definedName name="List_ModOutcomes">#REF!</definedName>
     <definedName name="List_ModTriggers">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <x:ext xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -170,16 +170,16 @@
     <t>form</t>
   </si>
   <si>
-    <t>string list</t>
-  </si>
-  <si>
-    <t>form list</t>
-  </si>
-  <si>
     <t>bool</t>
   </si>
   <si>
     <t>float</t>
+  </si>
+  <si>
+    <t>string[]</t>
+  </si>
+  <si>
+    <t>form[]</t>
   </si>
 </sst>
 </file>
@@ -894,17 +894,17 @@
         <v>44</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="6" t="s">
         <v>44</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q5" s="6" t="s">
         <v>44</v>
@@ -955,31 +955,31 @@
         <v>45</v>
       </c>
       <c r="AG5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AJ5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AL5" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="AH5" s="6" t="s">
+      <c r="AN5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="AI5" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ5" s="6" t="s">
+      <c r="AO5" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="AK5" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="AL5" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="AM5" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="AN5" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="AO5" s="6" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="6" spans="2:41" s="2" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>